<commit_message>
Full system sync from 📦 Warehouse Operations
</commit_message>
<xml_diff>
--- a/03_Procurement_Supply_Stock_Alert.xlsx
+++ b/03_Procurement_Supply_Stock_Alert.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-23 16:43</t>
+          <t>2026-09-23 16:44</t>
         </is>
       </c>
       <c r="R2" t="inlineStr"/>
@@ -723,7 +723,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-23 16:43</t>
+          <t>2026-09-23 16:44</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
@@ -802,7 +802,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-23 16:43</t>
+          <t>2026-09-23 16:44</t>
         </is>
       </c>
       <c r="R4" t="inlineStr"/>

</xml_diff>